<commit_message>
Pair game: pair videos by the sheet's Pair ID, add the vlogger clips
real_vs_ai_videos_3.xlsx adds a Pair ID column and a real + AI vlogger pair. Every video
in videos.json now has a pair number; getFixedPairs (dataset/loader.js) joins a real and
an AI clip with the same number, and each game shows two of these pairs (rounds 4 and 7).
Tests check that every Pair ID has exactly one real and one AI clip. The new sheet
replaces content/videos/real_vs_ai_videos.xlsx (same rows plus the new ones).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/videos/real_vs_ai_videos.xlsx
+++ b/content/videos/real_vs_ai_videos.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Videos!$A$1:$E$201</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Videos!$A$1:$F$201</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="45">
   <si>
     <t xml:space="preserve">Video</t>
   </si>
@@ -41,6 +41,9 @@
     <t xml:space="preserve">Real or AI</t>
   </si>
   <si>
+    <t xml:space="preserve">Pair ID</t>
+  </si>
+  <si>
     <t xml:space="preserve">Person flipping through a book</t>
   </si>
   <si>
@@ -95,6 +98,30 @@
     <t xml:space="preserve">Pair with the real book-flipping clip. Clues: text on pages warping or turning to gibberish, pages merging or bending oddly, extra or missing fingers</t>
   </si>
   <si>
+    <t xml:space="preserve">Vlogger speaking to camera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://canva.link/eejyx94bum8pdbv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A real vlogger talking directly to the camera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clues: natural blinking and eye movement, lips match speech, background stays consistent, natural hand gestures</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI vlogger speaking to camera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://canva.link/xl4p0kvnk3abq24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI-generated vlogger talking directly to the camera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pair with the real vlogger clip. Clues: unnatural or missing blinking, lips slightly out of sync, overly smooth skin, background objects shifting, stiff or repetitive gestures</t>
+  </si>
+  <si>
     <t xml:space="preserve">How to use this sheet</t>
   </si>
   <si>
@@ -117,6 +144,9 @@
   </si>
   <si>
     <t xml:space="preserve">Add each new video on the next empty row of the Videos tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same number on a Real and an AI video = shown side by side (e.g. 1 and 1)</t>
   </si>
   <si>
     <t xml:space="preserve">Summary</t>
@@ -138,7 +168,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -192,6 +222,13 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -268,7 +305,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -306,6 +343,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -642,7 +687,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E201"/>
+  <dimension ref="A1:F201"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
@@ -650,6 +695,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="50"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -668,88 +714,129 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="5"/>
+      <c r="A6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="5"/>
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3"/>
@@ -757,6 +844,7 @@
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3"/>
@@ -764,6 +852,7 @@
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3"/>
@@ -771,6 +860,7 @@
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3"/>
@@ -778,6 +868,7 @@
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3"/>
@@ -785,6 +876,7 @@
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3"/>
@@ -792,6 +884,7 @@
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3"/>
@@ -799,6 +892,7 @@
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
       <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3"/>
@@ -806,6 +900,7 @@
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
       <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3"/>
@@ -813,6 +908,7 @@
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
       <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3"/>
@@ -820,6 +916,7 @@
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3"/>
@@ -827,6 +924,7 @@
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
       <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3"/>
@@ -834,6 +932,7 @@
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
       <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3"/>
@@ -841,6 +940,7 @@
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
       <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3"/>
@@ -848,6 +948,7 @@
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
       <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3"/>
@@ -855,6 +956,7 @@
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
       <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3"/>
@@ -862,6 +964,7 @@
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
       <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3"/>
@@ -869,6 +972,7 @@
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
       <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3"/>
@@ -876,6 +980,7 @@
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
       <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3"/>
@@ -883,6 +988,7 @@
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
       <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="3"/>
@@ -890,6 +996,7 @@
       <c r="C27" s="4"/>
       <c r="D27" s="4"/>
       <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3"/>
@@ -897,6 +1004,7 @@
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
       <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="3"/>
@@ -904,6 +1012,7 @@
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
       <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3"/>
@@ -911,6 +1020,7 @@
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
       <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="3"/>
@@ -918,6 +1028,7 @@
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
       <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="3"/>
@@ -925,6 +1036,7 @@
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
       <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3"/>
@@ -932,6 +1044,7 @@
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
       <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3"/>
@@ -939,6 +1052,7 @@
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
       <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="3"/>
@@ -946,6 +1060,7 @@
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
       <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3"/>
@@ -953,6 +1068,7 @@
       <c r="C36" s="4"/>
       <c r="D36" s="4"/>
       <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="3"/>
@@ -960,6 +1076,7 @@
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
       <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3"/>
@@ -967,6 +1084,7 @@
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
       <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="3"/>
@@ -974,6 +1092,7 @@
       <c r="C39" s="4"/>
       <c r="D39" s="4"/>
       <c r="E39" s="5"/>
+      <c r="F39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3"/>
@@ -981,6 +1100,7 @@
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
       <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="3"/>
@@ -988,6 +1108,7 @@
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
       <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3"/>
@@ -995,6 +1116,7 @@
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
       <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="3"/>
@@ -1002,6 +1124,7 @@
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
       <c r="E43" s="5"/>
+      <c r="F43" s="5"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="3"/>
@@ -1009,6 +1132,7 @@
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
       <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="3"/>
@@ -1016,6 +1140,7 @@
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
       <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3"/>
@@ -1023,6 +1148,7 @@
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
       <c r="E46" s="5"/>
+      <c r="F46" s="5"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="3"/>
@@ -1030,6 +1156,7 @@
       <c r="C47" s="4"/>
       <c r="D47" s="4"/>
       <c r="E47" s="5"/>
+      <c r="F47" s="5"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="3"/>
@@ -1037,6 +1164,7 @@
       <c r="C48" s="4"/>
       <c r="D48" s="4"/>
       <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="3"/>
@@ -1044,6 +1172,7 @@
       <c r="C49" s="4"/>
       <c r="D49" s="4"/>
       <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="3"/>
@@ -1051,6 +1180,7 @@
       <c r="C50" s="4"/>
       <c r="D50" s="4"/>
       <c r="E50" s="5"/>
+      <c r="F50" s="5"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="3"/>
@@ -1058,6 +1188,7 @@
       <c r="C51" s="4"/>
       <c r="D51" s="4"/>
       <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="3"/>
@@ -1065,6 +1196,7 @@
       <c r="C52" s="4"/>
       <c r="D52" s="4"/>
       <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="3"/>
@@ -1072,6 +1204,7 @@
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
       <c r="E53" s="5"/>
+      <c r="F53" s="5"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="3"/>
@@ -1079,6 +1212,7 @@
       <c r="C54" s="4"/>
       <c r="D54" s="4"/>
       <c r="E54" s="5"/>
+      <c r="F54" s="5"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="3"/>
@@ -1086,6 +1220,7 @@
       <c r="C55" s="4"/>
       <c r="D55" s="4"/>
       <c r="E55" s="5"/>
+      <c r="F55" s="5"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="3"/>
@@ -1093,6 +1228,7 @@
       <c r="C56" s="4"/>
       <c r="D56" s="4"/>
       <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="3"/>
@@ -1100,6 +1236,7 @@
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="3"/>
@@ -1107,6 +1244,7 @@
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="5"/>
+      <c r="F58" s="5"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="3"/>
@@ -1114,6 +1252,7 @@
       <c r="C59" s="4"/>
       <c r="D59" s="4"/>
       <c r="E59" s="5"/>
+      <c r="F59" s="5"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="3"/>
@@ -1121,6 +1260,7 @@
       <c r="C60" s="4"/>
       <c r="D60" s="4"/>
       <c r="E60" s="5"/>
+      <c r="F60" s="5"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="3"/>
@@ -1128,6 +1268,7 @@
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="3"/>
@@ -1135,6 +1276,7 @@
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
       <c r="E62" s="5"/>
+      <c r="F62" s="5"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="3"/>
@@ -1142,6 +1284,7 @@
       <c r="C63" s="4"/>
       <c r="D63" s="4"/>
       <c r="E63" s="5"/>
+      <c r="F63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="3"/>
@@ -1149,6 +1292,7 @@
       <c r="C64" s="4"/>
       <c r="D64" s="4"/>
       <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="3"/>
@@ -1156,6 +1300,7 @@
       <c r="C65" s="4"/>
       <c r="D65" s="4"/>
       <c r="E65" s="5"/>
+      <c r="F65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="3"/>
@@ -1163,6 +1308,7 @@
       <c r="C66" s="4"/>
       <c r="D66" s="4"/>
       <c r="E66" s="5"/>
+      <c r="F66" s="5"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="3"/>
@@ -1170,6 +1316,7 @@
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
       <c r="E67" s="5"/>
+      <c r="F67" s="5"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3"/>
@@ -1177,6 +1324,7 @@
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
       <c r="E68" s="5"/>
+      <c r="F68" s="5"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="3"/>
@@ -1184,6 +1332,7 @@
       <c r="C69" s="4"/>
       <c r="D69" s="4"/>
       <c r="E69" s="5"/>
+      <c r="F69" s="5"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3"/>
@@ -1191,6 +1340,7 @@
       <c r="C70" s="4"/>
       <c r="D70" s="4"/>
       <c r="E70" s="5"/>
+      <c r="F70" s="5"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="3"/>
@@ -1198,6 +1348,7 @@
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
       <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3"/>
@@ -1205,6 +1356,7 @@
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
       <c r="E72" s="5"/>
+      <c r="F72" s="5"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="3"/>
@@ -1212,6 +1364,7 @@
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
       <c r="E73" s="5"/>
+      <c r="F73" s="5"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="3"/>
@@ -1219,6 +1372,7 @@
       <c r="C74" s="4"/>
       <c r="D74" s="4"/>
       <c r="E74" s="5"/>
+      <c r="F74" s="5"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="3"/>
@@ -1226,6 +1380,7 @@
       <c r="C75" s="4"/>
       <c r="D75" s="4"/>
       <c r="E75" s="5"/>
+      <c r="F75" s="5"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="3"/>
@@ -1233,6 +1388,7 @@
       <c r="C76" s="4"/>
       <c r="D76" s="4"/>
       <c r="E76" s="5"/>
+      <c r="F76" s="5"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="3"/>
@@ -1240,6 +1396,7 @@
       <c r="C77" s="4"/>
       <c r="D77" s="4"/>
       <c r="E77" s="5"/>
+      <c r="F77" s="5"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="3"/>
@@ -1247,6 +1404,7 @@
       <c r="C78" s="4"/>
       <c r="D78" s="4"/>
       <c r="E78" s="5"/>
+      <c r="F78" s="5"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="3"/>
@@ -1254,6 +1412,7 @@
       <c r="C79" s="4"/>
       <c r="D79" s="4"/>
       <c r="E79" s="5"/>
+      <c r="F79" s="5"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="3"/>
@@ -1261,6 +1420,7 @@
       <c r="C80" s="4"/>
       <c r="D80" s="4"/>
       <c r="E80" s="5"/>
+      <c r="F80" s="5"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="3"/>
@@ -1268,6 +1428,7 @@
       <c r="C81" s="4"/>
       <c r="D81" s="4"/>
       <c r="E81" s="5"/>
+      <c r="F81" s="5"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="3"/>
@@ -1275,6 +1436,7 @@
       <c r="C82" s="4"/>
       <c r="D82" s="4"/>
       <c r="E82" s="5"/>
+      <c r="F82" s="5"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="3"/>
@@ -1282,6 +1444,7 @@
       <c r="C83" s="4"/>
       <c r="D83" s="4"/>
       <c r="E83" s="5"/>
+      <c r="F83" s="5"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="3"/>
@@ -1289,6 +1452,7 @@
       <c r="C84" s="4"/>
       <c r="D84" s="4"/>
       <c r="E84" s="5"/>
+      <c r="F84" s="5"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="3"/>
@@ -1296,6 +1460,7 @@
       <c r="C85" s="4"/>
       <c r="D85" s="4"/>
       <c r="E85" s="5"/>
+      <c r="F85" s="5"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="3"/>
@@ -1303,6 +1468,7 @@
       <c r="C86" s="4"/>
       <c r="D86" s="4"/>
       <c r="E86" s="5"/>
+      <c r="F86" s="5"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="3"/>
@@ -1310,6 +1476,7 @@
       <c r="C87" s="4"/>
       <c r="D87" s="4"/>
       <c r="E87" s="5"/>
+      <c r="F87" s="5"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="3"/>
@@ -1317,6 +1484,7 @@
       <c r="C88" s="4"/>
       <c r="D88" s="4"/>
       <c r="E88" s="5"/>
+      <c r="F88" s="5"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="3"/>
@@ -1324,6 +1492,7 @@
       <c r="C89" s="4"/>
       <c r="D89" s="4"/>
       <c r="E89" s="5"/>
+      <c r="F89" s="5"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="3"/>
@@ -1331,6 +1500,7 @@
       <c r="C90" s="4"/>
       <c r="D90" s="4"/>
       <c r="E90" s="5"/>
+      <c r="F90" s="5"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="3"/>
@@ -1338,6 +1508,7 @@
       <c r="C91" s="4"/>
       <c r="D91" s="4"/>
       <c r="E91" s="5"/>
+      <c r="F91" s="5"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="3"/>
@@ -1345,6 +1516,7 @@
       <c r="C92" s="4"/>
       <c r="D92" s="4"/>
       <c r="E92" s="5"/>
+      <c r="F92" s="5"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="3"/>
@@ -1352,6 +1524,7 @@
       <c r="C93" s="4"/>
       <c r="D93" s="4"/>
       <c r="E93" s="5"/>
+      <c r="F93" s="5"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="3"/>
@@ -1359,6 +1532,7 @@
       <c r="C94" s="4"/>
       <c r="D94" s="4"/>
       <c r="E94" s="5"/>
+      <c r="F94" s="5"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="3"/>
@@ -1366,6 +1540,7 @@
       <c r="C95" s="4"/>
       <c r="D95" s="4"/>
       <c r="E95" s="5"/>
+      <c r="F95" s="5"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="3"/>
@@ -1373,6 +1548,7 @@
       <c r="C96" s="4"/>
       <c r="D96" s="4"/>
       <c r="E96" s="5"/>
+      <c r="F96" s="5"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="3"/>
@@ -1380,6 +1556,7 @@
       <c r="C97" s="4"/>
       <c r="D97" s="4"/>
       <c r="E97" s="5"/>
+      <c r="F97" s="5"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="3"/>
@@ -1387,6 +1564,7 @@
       <c r="C98" s="4"/>
       <c r="D98" s="4"/>
       <c r="E98" s="5"/>
+      <c r="F98" s="5"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="3"/>
@@ -1394,6 +1572,7 @@
       <c r="C99" s="4"/>
       <c r="D99" s="4"/>
       <c r="E99" s="5"/>
+      <c r="F99" s="5"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="3"/>
@@ -1401,6 +1580,7 @@
       <c r="C100" s="4"/>
       <c r="D100" s="4"/>
       <c r="E100" s="5"/>
+      <c r="F100" s="5"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="3"/>
@@ -1408,6 +1588,7 @@
       <c r="C101" s="4"/>
       <c r="D101" s="4"/>
       <c r="E101" s="5"/>
+      <c r="F101" s="5"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="3"/>
@@ -1415,6 +1596,7 @@
       <c r="C102" s="4"/>
       <c r="D102" s="4"/>
       <c r="E102" s="5"/>
+      <c r="F102" s="5"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="3"/>
@@ -1422,6 +1604,7 @@
       <c r="C103" s="4"/>
       <c r="D103" s="4"/>
       <c r="E103" s="5"/>
+      <c r="F103" s="5"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="3"/>
@@ -1429,6 +1612,7 @@
       <c r="C104" s="4"/>
       <c r="D104" s="4"/>
       <c r="E104" s="5"/>
+      <c r="F104" s="5"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="3"/>
@@ -1436,6 +1620,7 @@
       <c r="C105" s="4"/>
       <c r="D105" s="4"/>
       <c r="E105" s="5"/>
+      <c r="F105" s="5"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="3"/>
@@ -1443,6 +1628,7 @@
       <c r="C106" s="4"/>
       <c r="D106" s="4"/>
       <c r="E106" s="5"/>
+      <c r="F106" s="5"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="3"/>
@@ -1450,6 +1636,7 @@
       <c r="C107" s="4"/>
       <c r="D107" s="4"/>
       <c r="E107" s="5"/>
+      <c r="F107" s="5"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="3"/>
@@ -1457,6 +1644,7 @@
       <c r="C108" s="4"/>
       <c r="D108" s="4"/>
       <c r="E108" s="5"/>
+      <c r="F108" s="5"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="3"/>
@@ -1464,6 +1652,7 @@
       <c r="C109" s="4"/>
       <c r="D109" s="4"/>
       <c r="E109" s="5"/>
+      <c r="F109" s="5"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="3"/>
@@ -1471,6 +1660,7 @@
       <c r="C110" s="4"/>
       <c r="D110" s="4"/>
       <c r="E110" s="5"/>
+      <c r="F110" s="5"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="3"/>
@@ -1478,6 +1668,7 @@
       <c r="C111" s="4"/>
       <c r="D111" s="4"/>
       <c r="E111" s="5"/>
+      <c r="F111" s="5"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="3"/>
@@ -1485,6 +1676,7 @@
       <c r="C112" s="4"/>
       <c r="D112" s="4"/>
       <c r="E112" s="5"/>
+      <c r="F112" s="5"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="3"/>
@@ -1492,6 +1684,7 @@
       <c r="C113" s="4"/>
       <c r="D113" s="4"/>
       <c r="E113" s="5"/>
+      <c r="F113" s="5"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="3"/>
@@ -1499,6 +1692,7 @@
       <c r="C114" s="4"/>
       <c r="D114" s="4"/>
       <c r="E114" s="5"/>
+      <c r="F114" s="5"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="3"/>
@@ -1506,6 +1700,7 @@
       <c r="C115" s="4"/>
       <c r="D115" s="4"/>
       <c r="E115" s="5"/>
+      <c r="F115" s="5"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="3"/>
@@ -1513,6 +1708,7 @@
       <c r="C116" s="4"/>
       <c r="D116" s="4"/>
       <c r="E116" s="5"/>
+      <c r="F116" s="5"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="3"/>
@@ -1520,6 +1716,7 @@
       <c r="C117" s="4"/>
       <c r="D117" s="4"/>
       <c r="E117" s="5"/>
+      <c r="F117" s="5"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="3"/>
@@ -1527,6 +1724,7 @@
       <c r="C118" s="4"/>
       <c r="D118" s="4"/>
       <c r="E118" s="5"/>
+      <c r="F118" s="5"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="3"/>
@@ -1534,6 +1732,7 @@
       <c r="C119" s="4"/>
       <c r="D119" s="4"/>
       <c r="E119" s="5"/>
+      <c r="F119" s="5"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="3"/>
@@ -1541,6 +1740,7 @@
       <c r="C120" s="4"/>
       <c r="D120" s="4"/>
       <c r="E120" s="5"/>
+      <c r="F120" s="5"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="3"/>
@@ -1548,6 +1748,7 @@
       <c r="C121" s="4"/>
       <c r="D121" s="4"/>
       <c r="E121" s="5"/>
+      <c r="F121" s="5"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="3"/>
@@ -1555,6 +1756,7 @@
       <c r="C122" s="4"/>
       <c r="D122" s="4"/>
       <c r="E122" s="5"/>
+      <c r="F122" s="5"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="3"/>
@@ -1562,6 +1764,7 @@
       <c r="C123" s="4"/>
       <c r="D123" s="4"/>
       <c r="E123" s="5"/>
+      <c r="F123" s="5"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="3"/>
@@ -1569,6 +1772,7 @@
       <c r="C124" s="4"/>
       <c r="D124" s="4"/>
       <c r="E124" s="5"/>
+      <c r="F124" s="5"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="3"/>
@@ -1576,6 +1780,7 @@
       <c r="C125" s="4"/>
       <c r="D125" s="4"/>
       <c r="E125" s="5"/>
+      <c r="F125" s="5"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="3"/>
@@ -1583,6 +1788,7 @@
       <c r="C126" s="4"/>
       <c r="D126" s="4"/>
       <c r="E126" s="5"/>
+      <c r="F126" s="5"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="3"/>
@@ -1590,6 +1796,7 @@
       <c r="C127" s="4"/>
       <c r="D127" s="4"/>
       <c r="E127" s="5"/>
+      <c r="F127" s="5"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="3"/>
@@ -1597,6 +1804,7 @@
       <c r="C128" s="4"/>
       <c r="D128" s="4"/>
       <c r="E128" s="5"/>
+      <c r="F128" s="5"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="3"/>
@@ -1604,6 +1812,7 @@
       <c r="C129" s="4"/>
       <c r="D129" s="4"/>
       <c r="E129" s="5"/>
+      <c r="F129" s="5"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="3"/>
@@ -1611,6 +1820,7 @@
       <c r="C130" s="4"/>
       <c r="D130" s="4"/>
       <c r="E130" s="5"/>
+      <c r="F130" s="5"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="3"/>
@@ -1618,6 +1828,7 @@
       <c r="C131" s="4"/>
       <c r="D131" s="4"/>
       <c r="E131" s="5"/>
+      <c r="F131" s="5"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="3"/>
@@ -1625,6 +1836,7 @@
       <c r="C132" s="4"/>
       <c r="D132" s="4"/>
       <c r="E132" s="5"/>
+      <c r="F132" s="5"/>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="3"/>
@@ -1632,6 +1844,7 @@
       <c r="C133" s="4"/>
       <c r="D133" s="4"/>
       <c r="E133" s="5"/>
+      <c r="F133" s="5"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="3"/>
@@ -1639,6 +1852,7 @@
       <c r="C134" s="4"/>
       <c r="D134" s="4"/>
       <c r="E134" s="5"/>
+      <c r="F134" s="5"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="3"/>
@@ -1646,6 +1860,7 @@
       <c r="C135" s="4"/>
       <c r="D135" s="4"/>
       <c r="E135" s="5"/>
+      <c r="F135" s="5"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="3"/>
@@ -1653,6 +1868,7 @@
       <c r="C136" s="4"/>
       <c r="D136" s="4"/>
       <c r="E136" s="5"/>
+      <c r="F136" s="5"/>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="3"/>
@@ -1660,6 +1876,7 @@
       <c r="C137" s="4"/>
       <c r="D137" s="4"/>
       <c r="E137" s="5"/>
+      <c r="F137" s="5"/>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="3"/>
@@ -1667,6 +1884,7 @@
       <c r="C138" s="4"/>
       <c r="D138" s="4"/>
       <c r="E138" s="5"/>
+      <c r="F138" s="5"/>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="3"/>
@@ -1674,6 +1892,7 @@
       <c r="C139" s="4"/>
       <c r="D139" s="4"/>
       <c r="E139" s="5"/>
+      <c r="F139" s="5"/>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="3"/>
@@ -1681,6 +1900,7 @@
       <c r="C140" s="4"/>
       <c r="D140" s="4"/>
       <c r="E140" s="5"/>
+      <c r="F140" s="5"/>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="3"/>
@@ -1688,6 +1908,7 @@
       <c r="C141" s="4"/>
       <c r="D141" s="4"/>
       <c r="E141" s="5"/>
+      <c r="F141" s="5"/>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="3"/>
@@ -1695,6 +1916,7 @@
       <c r="C142" s="4"/>
       <c r="D142" s="4"/>
       <c r="E142" s="5"/>
+      <c r="F142" s="5"/>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="3"/>
@@ -1702,6 +1924,7 @@
       <c r="C143" s="4"/>
       <c r="D143" s="4"/>
       <c r="E143" s="5"/>
+      <c r="F143" s="5"/>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="3"/>
@@ -1709,6 +1932,7 @@
       <c r="C144" s="4"/>
       <c r="D144" s="4"/>
       <c r="E144" s="5"/>
+      <c r="F144" s="5"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="3"/>
@@ -1716,6 +1940,7 @@
       <c r="C145" s="4"/>
       <c r="D145" s="4"/>
       <c r="E145" s="5"/>
+      <c r="F145" s="5"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="3"/>
@@ -1723,6 +1948,7 @@
       <c r="C146" s="4"/>
       <c r="D146" s="4"/>
       <c r="E146" s="5"/>
+      <c r="F146" s="5"/>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="3"/>
@@ -1730,6 +1956,7 @@
       <c r="C147" s="4"/>
       <c r="D147" s="4"/>
       <c r="E147" s="5"/>
+      <c r="F147" s="5"/>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="3"/>
@@ -1737,6 +1964,7 @@
       <c r="C148" s="4"/>
       <c r="D148" s="4"/>
       <c r="E148" s="5"/>
+      <c r="F148" s="5"/>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="3"/>
@@ -1744,6 +1972,7 @@
       <c r="C149" s="4"/>
       <c r="D149" s="4"/>
       <c r="E149" s="5"/>
+      <c r="F149" s="5"/>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="3"/>
@@ -1751,6 +1980,7 @@
       <c r="C150" s="4"/>
       <c r="D150" s="4"/>
       <c r="E150" s="5"/>
+      <c r="F150" s="5"/>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="3"/>
@@ -1758,6 +1988,7 @@
       <c r="C151" s="4"/>
       <c r="D151" s="4"/>
       <c r="E151" s="5"/>
+      <c r="F151" s="5"/>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="3"/>
@@ -1765,6 +1996,7 @@
       <c r="C152" s="4"/>
       <c r="D152" s="4"/>
       <c r="E152" s="5"/>
+      <c r="F152" s="5"/>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="3"/>
@@ -1772,6 +2004,7 @@
       <c r="C153" s="4"/>
       <c r="D153" s="4"/>
       <c r="E153" s="5"/>
+      <c r="F153" s="5"/>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="3"/>
@@ -1779,6 +2012,7 @@
       <c r="C154" s="4"/>
       <c r="D154" s="4"/>
       <c r="E154" s="5"/>
+      <c r="F154" s="5"/>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="3"/>
@@ -1786,6 +2020,7 @@
       <c r="C155" s="4"/>
       <c r="D155" s="4"/>
       <c r="E155" s="5"/>
+      <c r="F155" s="5"/>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="3"/>
@@ -1793,6 +2028,7 @@
       <c r="C156" s="4"/>
       <c r="D156" s="4"/>
       <c r="E156" s="5"/>
+      <c r="F156" s="5"/>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="3"/>
@@ -1800,6 +2036,7 @@
       <c r="C157" s="4"/>
       <c r="D157" s="4"/>
       <c r="E157" s="5"/>
+      <c r="F157" s="5"/>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="3"/>
@@ -1807,6 +2044,7 @@
       <c r="C158" s="4"/>
       <c r="D158" s="4"/>
       <c r="E158" s="5"/>
+      <c r="F158" s="5"/>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="3"/>
@@ -1814,6 +2052,7 @@
       <c r="C159" s="4"/>
       <c r="D159" s="4"/>
       <c r="E159" s="5"/>
+      <c r="F159" s="5"/>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="3"/>
@@ -1821,6 +2060,7 @@
       <c r="C160" s="4"/>
       <c r="D160" s="4"/>
       <c r="E160" s="5"/>
+      <c r="F160" s="5"/>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="3"/>
@@ -1828,6 +2068,7 @@
       <c r="C161" s="4"/>
       <c r="D161" s="4"/>
       <c r="E161" s="5"/>
+      <c r="F161" s="5"/>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="3"/>
@@ -1835,6 +2076,7 @@
       <c r="C162" s="4"/>
       <c r="D162" s="4"/>
       <c r="E162" s="5"/>
+      <c r="F162" s="5"/>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="3"/>
@@ -1842,6 +2084,7 @@
       <c r="C163" s="4"/>
       <c r="D163" s="4"/>
       <c r="E163" s="5"/>
+      <c r="F163" s="5"/>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="3"/>
@@ -1849,6 +2092,7 @@
       <c r="C164" s="4"/>
       <c r="D164" s="4"/>
       <c r="E164" s="5"/>
+      <c r="F164" s="5"/>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="3"/>
@@ -1856,6 +2100,7 @@
       <c r="C165" s="4"/>
       <c r="D165" s="4"/>
       <c r="E165" s="5"/>
+      <c r="F165" s="5"/>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="3"/>
@@ -1863,6 +2108,7 @@
       <c r="C166" s="4"/>
       <c r="D166" s="4"/>
       <c r="E166" s="5"/>
+      <c r="F166" s="5"/>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="3"/>
@@ -1870,6 +2116,7 @@
       <c r="C167" s="4"/>
       <c r="D167" s="4"/>
       <c r="E167" s="5"/>
+      <c r="F167" s="5"/>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="3"/>
@@ -1877,6 +2124,7 @@
       <c r="C168" s="4"/>
       <c r="D168" s="4"/>
       <c r="E168" s="5"/>
+      <c r="F168" s="5"/>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="3"/>
@@ -1884,6 +2132,7 @@
       <c r="C169" s="4"/>
       <c r="D169" s="4"/>
       <c r="E169" s="5"/>
+      <c r="F169" s="5"/>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="3"/>
@@ -1891,6 +2140,7 @@
       <c r="C170" s="4"/>
       <c r="D170" s="4"/>
       <c r="E170" s="5"/>
+      <c r="F170" s="5"/>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="3"/>
@@ -1898,6 +2148,7 @@
       <c r="C171" s="4"/>
       <c r="D171" s="4"/>
       <c r="E171" s="5"/>
+      <c r="F171" s="5"/>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="3"/>
@@ -1905,6 +2156,7 @@
       <c r="C172" s="4"/>
       <c r="D172" s="4"/>
       <c r="E172" s="5"/>
+      <c r="F172" s="5"/>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="3"/>
@@ -1912,6 +2164,7 @@
       <c r="C173" s="4"/>
       <c r="D173" s="4"/>
       <c r="E173" s="5"/>
+      <c r="F173" s="5"/>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="3"/>
@@ -1919,6 +2172,7 @@
       <c r="C174" s="4"/>
       <c r="D174" s="4"/>
       <c r="E174" s="5"/>
+      <c r="F174" s="5"/>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="3"/>
@@ -1926,6 +2180,7 @@
       <c r="C175" s="4"/>
       <c r="D175" s="4"/>
       <c r="E175" s="5"/>
+      <c r="F175" s="5"/>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="3"/>
@@ -1933,6 +2188,7 @@
       <c r="C176" s="4"/>
       <c r="D176" s="4"/>
       <c r="E176" s="5"/>
+      <c r="F176" s="5"/>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="3"/>
@@ -1940,6 +2196,7 @@
       <c r="C177" s="4"/>
       <c r="D177" s="4"/>
       <c r="E177" s="5"/>
+      <c r="F177" s="5"/>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="3"/>
@@ -1947,6 +2204,7 @@
       <c r="C178" s="4"/>
       <c r="D178" s="4"/>
       <c r="E178" s="5"/>
+      <c r="F178" s="5"/>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="3"/>
@@ -1954,6 +2212,7 @@
       <c r="C179" s="4"/>
       <c r="D179" s="4"/>
       <c r="E179" s="5"/>
+      <c r="F179" s="5"/>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="3"/>
@@ -1961,6 +2220,7 @@
       <c r="C180" s="4"/>
       <c r="D180" s="4"/>
       <c r="E180" s="5"/>
+      <c r="F180" s="5"/>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="3"/>
@@ -1968,6 +2228,7 @@
       <c r="C181" s="4"/>
       <c r="D181" s="4"/>
       <c r="E181" s="5"/>
+      <c r="F181" s="5"/>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A182" s="3"/>
@@ -1975,6 +2236,7 @@
       <c r="C182" s="4"/>
       <c r="D182" s="4"/>
       <c r="E182" s="5"/>
+      <c r="F182" s="5"/>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A183" s="3"/>
@@ -1982,6 +2244,7 @@
       <c r="C183" s="4"/>
       <c r="D183" s="4"/>
       <c r="E183" s="5"/>
+      <c r="F183" s="5"/>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A184" s="3"/>
@@ -1989,6 +2252,7 @@
       <c r="C184" s="4"/>
       <c r="D184" s="4"/>
       <c r="E184" s="5"/>
+      <c r="F184" s="5"/>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A185" s="3"/>
@@ -1996,6 +2260,7 @@
       <c r="C185" s="4"/>
       <c r="D185" s="4"/>
       <c r="E185" s="5"/>
+      <c r="F185" s="5"/>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A186" s="3"/>
@@ -2003,6 +2268,7 @@
       <c r="C186" s="4"/>
       <c r="D186" s="4"/>
       <c r="E186" s="5"/>
+      <c r="F186" s="5"/>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A187" s="3"/>
@@ -2010,6 +2276,7 @@
       <c r="C187" s="4"/>
       <c r="D187" s="4"/>
       <c r="E187" s="5"/>
+      <c r="F187" s="5"/>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A188" s="3"/>
@@ -2017,6 +2284,7 @@
       <c r="C188" s="4"/>
       <c r="D188" s="4"/>
       <c r="E188" s="5"/>
+      <c r="F188" s="5"/>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A189" s="3"/>
@@ -2024,6 +2292,7 @@
       <c r="C189" s="4"/>
       <c r="D189" s="4"/>
       <c r="E189" s="5"/>
+      <c r="F189" s="5"/>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A190" s="3"/>
@@ -2031,6 +2300,7 @@
       <c r="C190" s="4"/>
       <c r="D190" s="4"/>
       <c r="E190" s="5"/>
+      <c r="F190" s="5"/>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A191" s="3"/>
@@ -2038,6 +2308,7 @@
       <c r="C191" s="4"/>
       <c r="D191" s="4"/>
       <c r="E191" s="5"/>
+      <c r="F191" s="5"/>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A192" s="3"/>
@@ -2045,6 +2316,7 @@
       <c r="C192" s="4"/>
       <c r="D192" s="4"/>
       <c r="E192" s="5"/>
+      <c r="F192" s="5"/>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A193" s="3"/>
@@ -2052,6 +2324,7 @@
       <c r="C193" s="4"/>
       <c r="D193" s="4"/>
       <c r="E193" s="5"/>
+      <c r="F193" s="5"/>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A194" s="3"/>
@@ -2059,6 +2332,7 @@
       <c r="C194" s="4"/>
       <c r="D194" s="4"/>
       <c r="E194" s="5"/>
+      <c r="F194" s="5"/>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A195" s="3"/>
@@ -2066,6 +2340,7 @@
       <c r="C195" s="4"/>
       <c r="D195" s="4"/>
       <c r="E195" s="5"/>
+      <c r="F195" s="5"/>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A196" s="3"/>
@@ -2073,6 +2348,7 @@
       <c r="C196" s="4"/>
       <c r="D196" s="4"/>
       <c r="E196" s="5"/>
+      <c r="F196" s="5"/>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A197" s="3"/>
@@ -2080,6 +2356,7 @@
       <c r="C197" s="4"/>
       <c r="D197" s="4"/>
       <c r="E197" s="5"/>
+      <c r="F197" s="5"/>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A198" s="3"/>
@@ -2087,6 +2364,7 @@
       <c r="C198" s="4"/>
       <c r="D198" s="4"/>
       <c r="E198" s="5"/>
+      <c r="F198" s="5"/>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A199" s="3"/>
@@ -2094,6 +2372,7 @@
       <c r="C199" s="4"/>
       <c r="D199" s="4"/>
       <c r="E199" s="5"/>
+      <c r="F199" s="5"/>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A200" s="3"/>
@@ -2101,6 +2380,7 @@
       <c r="C200" s="4"/>
       <c r="D200" s="4"/>
       <c r="E200" s="5"/>
+      <c r="F200" s="5"/>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A201" s="3"/>
@@ -2108,9 +2388,10 @@
       <c r="C201" s="4"/>
       <c r="D201" s="4"/>
       <c r="E201" s="5"/>
+      <c r="F201" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E201"/>
+  <autoFilter ref="A1:F201"/>
   <conditionalFormatting sqref="E2:E201">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>$E2="Real"</formula>
@@ -2150,7 +2431,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="B1" s="7"/>
     </row>
@@ -2159,7 +2440,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2167,7 +2448,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2175,7 +2456,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2183,7 +2464,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2191,57 +2472,61 @@
         <v>4</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8"/>
-      <c r="B8" s="7"/>
+      <c r="A8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="B9" s="7"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">COUNTIF(Videos!E2:E201,"Real")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="B11" s="7" t="n">
         <f aca="false">COUNTIF(Videos!E2:E201,"AI")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B12" s="7" t="n">
         <f aca="false">B10+B11</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8"/>
-      <c r="B13" s="9"/>
+      <c r="B13" s="11"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>